<commit_message>
Add pre-filled Pattern of Study template, depersonalize the blank one
pattern_of_study_filled.xlsx has all 66 rows of currently-confirmed
pattern data (all 11 diploma programs, 26 AUT session), pulled directly
from pattern_table.json so it can't drift from what the tool actually
uses. The blank template's "Confirmed by Grant?" column is renamed to
"Confirmed?" to match the depersonalized wording used everywhere else.
</commit_message>
<xml_diff>
--- a/templates/pattern_of_study_template.xlsx
+++ b/templates/pattern_of_study_template.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Which position in that program's subject sequence, 1 and up. Positions 1-4 are confirmed to mean that season's Block 1-4. What positions 5+ mean is only empirically validated for diplomas (see the tool's pattern_lookup.py) - flag anything beyond position 4 as unconfirmed unless Grant has said otherwise for that specific case.</t>
+          <t>Which position in that program's subject sequence, 1 and up. Positions 1-4 are confirmed to mean that season's Block 1-4. What positions 5+ mean is only empirically validated for diplomas (see the tool's pattern_lookup.py) - flag anything beyond position 4 as unconfirmed unless it's been explicitly confirmed for that specific case.</t>
         </is>
       </c>
     </row>
@@ -545,12 +545,12 @@
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Confirmed by Grant?</t>
+          <t>Confirmed?</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Y if Grant has explicitly confirmed this exact row. N if it's your best inference from other data (e.g. a pattern you're fairly sure of but haven't had confirmed). This feeds the tool's confidence tiers - Y becomes "high" confidence, N stays "low" until confirmed.</t>
+          <t>Y if this exact row has been explicitly confirmed. N if it's your best inference from other data (e.g. a pattern you're fairly sure of but haven't had confirmed). This feeds the tool's confidence tiers - Y becomes "high" confidence, N stays "low" until confirmed.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Confirmed by Grant?</t>
+          <t>Confirmed?</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="1" ht="55" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>This sheet is intentionally empty. The tool's pattern reference data has zero prep-subject entries today (block subject codes only) - if you have the prep subject that should run for a given session/program (e.g. GEDU0016 / GEDU0017), fill it in below using the same confirmed-by-Grant convention as the Block Positions sheet.</t>
+          <t>This sheet is intentionally empty. The tool's pattern reference data has zero prep-subject entries today (block subject codes only) - if you have the prep subject that should run for a given session/program (e.g. GEDU0016 / GEDU0017), fill it in below using the same confirmed/not-confirmed convention as the Block Positions sheet.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Confirmed by Grant?</t>
+          <t>Confirmed?</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">

</xml_diff>